<commit_message>
Rebuild benchmark papers from scratch
</commit_message>
<xml_diff>
--- a/examples/real_cases/cumcm_2025_a/tables/data_profile/data_inventory.xlsx
+++ b/examples/real_cases/cumcm_2025_a/tables/data_profile/data_inventory.xlsx
@@ -666,7 +666,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>/Users/yangke/.codex/skills/guosai-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result1.xlsx</t>
+          <t>/Users/yangke/.codex/skills/cumcm-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result1.xlsx</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -717,7 +717,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>/Users/yangke/.codex/skills/guosai-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result2.xlsx</t>
+          <t>/Users/yangke/.codex/skills/cumcm-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result2.xlsx</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>/Users/yangke/.codex/skills/guosai-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result3.xlsx</t>
+          <t>/Users/yangke/.codex/skills/cumcm-math-modeling/examples/real_cases/cumcm_2025_a/data/raw/result3.xlsx</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>